<commit_message>
add measurement and update model of threaded rod
</commit_message>
<xml_diff>
--- a/Measurements/A5567820050 Drum clutch/v3/A5567820050.xlsx
+++ b/Measurements/A5567820050 Drum clutch/v3/A5567820050.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\solidworks\Measurements\A5567820050 Drum clutch\v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A15956E-B99C-4AD6-8027-A57979EFABE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE310A0B-21D9-405F-B515-10EC76E89827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{32BFC42B-CD3D-49FE-8254-52B3F518DB85}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{32BFC42B-CD3D-49FE-8254-52B3F518DB85}"/>
   </bookViews>
   <sheets>
     <sheet name="FAI" sheetId="3" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Tolerance Table " sheetId="5" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">FAI!$A$1:$M$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">FAI!$A$7:$M$53</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Print Page 1'!$A$1:$J$45</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Print Page 2'!$A$1:$R$43</definedName>
   </definedNames>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="46">
   <si>
     <t>Customer</t>
   </si>
@@ -112,12 +112,6 @@
     <t>Overall Length</t>
   </si>
   <si>
-    <t>ID at Drum bottom</t>
-  </si>
-  <si>
-    <t>ID at 7.5mm from drum bottom</t>
-  </si>
-  <si>
     <t>Wall Thickness</t>
   </si>
   <si>
@@ -137,12 +131,6 @@
   </si>
   <si>
     <t>FAI</t>
-  </si>
-  <si>
-    <t>9a</t>
-  </si>
-  <si>
-    <t>9b</t>
   </si>
   <si>
     <t xml:space="preserve">Fillet Weld </t>
@@ -181,16 +169,22 @@
 5</t>
   </si>
   <si>
-    <t>Caliper?</t>
-  </si>
-  <si>
-    <t>???</t>
-  </si>
-  <si>
     <t>Meng</t>
   </si>
   <si>
     <t>02/23/2026</t>
+  </si>
+  <si>
+    <t>Micrometer</t>
+  </si>
+  <si>
+    <t>Caliper</t>
+  </si>
+  <si>
+    <t>Inner diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -787,9 +781,6 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="167" fontId="9" fillId="3" borderId="20" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -800,108 +791,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="9" fillId="3" borderId="21" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -1142,6 +1041,112 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="3" name="Straight Arrow Connector 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B4B06B4-D7FB-CC79-1469-50B33FB53A7D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="3143250" y="2571750"/>
+          <a:ext cx="66675" cy="771525"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>295275</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>523875</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="8" name="Straight Arrow Connector 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{39AFBC0C-4994-4443-8839-2507B48289F5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3952875" y="5238750"/>
+          <a:ext cx="228600" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent6"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent6"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent6"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1516,7 +1521,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" style="1" customWidth="1"/>
@@ -1537,17 +1542,17 @@
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="11" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D1" s="28"/>
       <c r="E1" s="40" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="G1" s="50" t="s">
-        <v>38</v>
+        <v>41</v>
+      </c>
+      <c r="G1" s="54" t="s">
+        <v>34</v>
       </c>
       <c r="H1" s="37"/>
       <c r="I1" s="31"/>
@@ -1564,7 +1569,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D2" s="29">
         <v>5</v>
@@ -1573,9 +1578,9 @@
         <v>4</v>
       </c>
       <c r="F2" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="G2" s="50"/>
+        <v>40</v>
+      </c>
+      <c r="G2" s="54"/>
       <c r="H2" s="38"/>
       <c r="I2" s="33"/>
       <c r="J2" s="33"/>
@@ -1592,7 +1597,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="42" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D3" s="30" t="s">
         <v>7</v>
@@ -1601,7 +1606,7 @@
         <v>8</v>
       </c>
       <c r="F3" s="27"/>
-      <c r="G3" s="50"/>
+      <c r="G3" s="54"/>
       <c r="H3" s="39"/>
       <c r="I3" s="35"/>
       <c r="J3" s="35"/>
@@ -1611,10 +1616,10 @@
     </row>
     <row r="4" spans="1:14" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="20" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C4" s="22" t="s">
         <v>9</v>
@@ -1634,23 +1639,23 @@
       <c r="H4" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="51" t="s">
+      <c r="I4" s="50" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="51" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="J4" s="52" t="s">
-        <v>40</v>
-      </c>
-      <c r="K4" s="52" t="s">
-        <v>41</v>
-      </c>
-      <c r="L4" s="53" t="s">
-        <v>42</v>
-      </c>
-      <c r="M4" s="54" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="L4" s="52" t="s">
+        <v>38</v>
+      </c>
+      <c r="M4" s="53" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="17">
         <v>1</v>
       </c>
@@ -1675,7 +1680,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I5" s="46"/>
       <c r="J5" s="46"/>
@@ -1683,7 +1688,7 @@
       <c r="L5" s="46"/>
       <c r="M5" s="46"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>2</v>
       </c>
@@ -1708,7 +1713,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I6" s="47"/>
       <c r="J6" s="47"/>
@@ -1733,23 +1738,33 @@
         <v>0</v>
       </c>
       <c r="F7" s="2">
-        <f t="shared" ref="F7:F26" si="0">C7+D7</f>
+        <f t="shared" ref="F7:F25" si="0">C7+D7</f>
         <v>50.1</v>
       </c>
       <c r="G7" s="2">
-        <f t="shared" ref="G7:G25" si="1">C7-E7</f>
+        <f t="shared" ref="G7:G24" si="1">C7-E7</f>
         <v>50</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="47"/>
-      <c r="J7" s="47"/>
-      <c r="K7" s="47"/>
-      <c r="L7" s="47"/>
-      <c r="M7" s="47"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I7" s="47">
+        <v>50.098700000000001</v>
+      </c>
+      <c r="J7" s="47">
+        <v>50.043500000000002</v>
+      </c>
+      <c r="K7" s="47">
+        <v>50.095199999999998</v>
+      </c>
+      <c r="L7" s="47">
+        <v>50.088700000000003</v>
+      </c>
+      <c r="M7" s="47">
+        <v>50.078099999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>4</v>
       </c>
@@ -1774,7 +1789,7 @@
         <v>16</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="I8" s="47"/>
       <c r="J8" s="47"/>
@@ -1807,13 +1822,23 @@
         <v>12</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="47"/>
-      <c r="J9" s="47"/>
-      <c r="K9" s="47"/>
-      <c r="L9" s="47"/>
-      <c r="M9" s="47"/>
+        <v>42</v>
+      </c>
+      <c r="I9" s="47">
+        <v>12.002000000000001</v>
+      </c>
+      <c r="J9" s="47">
+        <v>12.000999999999999</v>
+      </c>
+      <c r="K9" s="47">
+        <v>12.000999999999999</v>
+      </c>
+      <c r="L9" s="47">
+        <v>12.006</v>
+      </c>
+      <c r="M9" s="47">
+        <v>12.01</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
@@ -1840,13 +1865,23 @@
         <v>11.700000000000001</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I10" s="47"/>
-      <c r="J10" s="47"/>
-      <c r="K10" s="47"/>
-      <c r="L10" s="47"/>
-      <c r="M10" s="47"/>
+        <v>42</v>
+      </c>
+      <c r="I10" s="47">
+        <v>11.853</v>
+      </c>
+      <c r="J10" s="47">
+        <v>11.855</v>
+      </c>
+      <c r="K10" s="47">
+        <v>11.848000000000001</v>
+      </c>
+      <c r="L10" s="47">
+        <v>11.85</v>
+      </c>
+      <c r="M10" s="47">
+        <v>11.864000000000001</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
@@ -1875,11 +1910,21 @@
       <c r="H11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="47"/>
-      <c r="J11" s="47"/>
-      <c r="K11" s="47"/>
-      <c r="L11" s="47"/>
-      <c r="M11" s="47"/>
+      <c r="I11" s="47">
+        <v>9.9589999999999996</v>
+      </c>
+      <c r="J11" s="47">
+        <v>9.7055000000000007</v>
+      </c>
+      <c r="K11" s="47">
+        <v>10.116899999999999</v>
+      </c>
+      <c r="L11" s="47">
+        <v>10.337400000000001</v>
+      </c>
+      <c r="M11" s="47">
+        <v>10.545400000000001</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
@@ -1906,20 +1951,30 @@
         <v>68.5</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" s="47"/>
-      <c r="J12" s="47"/>
-      <c r="K12" s="47"/>
-      <c r="L12" s="47"/>
-      <c r="M12" s="47"/>
+        <v>43</v>
+      </c>
+      <c r="I12" s="47">
+        <v>68.87</v>
+      </c>
+      <c r="J12" s="47">
+        <v>69.19</v>
+      </c>
+      <c r="K12" s="47">
+        <v>68.98</v>
+      </c>
+      <c r="L12" s="47">
+        <v>69.19</v>
+      </c>
+      <c r="M12" s="47">
+        <v>69.48</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>31</v>
+      <c r="A13" s="4">
+        <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="C13" s="6">
         <v>50.3</v>
@@ -1938,305 +1993,395 @@
         <f t="shared" si="1"/>
         <v>49.599999999999994</v>
       </c>
-      <c r="H13" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="I13" s="47"/>
-      <c r="J13" s="47"/>
-      <c r="K13" s="47"/>
-      <c r="L13" s="47"/>
-      <c r="M13" s="47"/>
+      <c r="H13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I13" s="47">
+        <v>50.01</v>
+      </c>
+      <c r="J13" s="47">
+        <v>50.02</v>
+      </c>
+      <c r="K13" s="47">
+        <v>50.01</v>
+      </c>
+      <c r="L13" s="47">
+        <v>50.02</v>
+      </c>
+      <c r="M13" s="47">
+        <v>50.01</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>32</v>
+      <c r="A14" s="4">
+        <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C14" s="6">
-        <v>50.3</v>
+        <v>50</v>
       </c>
       <c r="D14" s="2">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="E14" s="2">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="F14" s="2">
         <f t="shared" si="0"/>
-        <v>51</v>
+        <v>50.1</v>
       </c>
       <c r="G14" s="2">
         <f t="shared" si="1"/>
-        <v>49.599999999999994</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I14" s="47"/>
-      <c r="J14" s="47"/>
-      <c r="K14" s="47"/>
-      <c r="L14" s="47"/>
-      <c r="M14" s="47"/>
+        <v>50</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I14" s="47">
+        <v>50.02</v>
+      </c>
+      <c r="J14" s="47">
+        <v>50.03</v>
+      </c>
+      <c r="K14" s="47">
+        <v>50.05</v>
+      </c>
+      <c r="L14" s="47">
+        <v>50.01</v>
+      </c>
+      <c r="M14" s="47">
+        <v>50.02</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C15" s="6">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="D15" s="2">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="E15" s="2">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="F15" s="2">
         <f t="shared" si="0"/>
-        <v>50.1</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="G15" s="2">
         <f t="shared" si="1"/>
-        <v>50</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="I15" s="47"/>
-      <c r="J15" s="47"/>
-      <c r="K15" s="47"/>
-      <c r="L15" s="47"/>
-      <c r="M15" s="47"/>
+        <v>1.7</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I15" s="47">
+        <v>2.0099999999999998</v>
+      </c>
+      <c r="J15" s="47">
+        <v>2.0299999999999998</v>
+      </c>
+      <c r="K15" s="47">
+        <v>2.0099999999999998</v>
+      </c>
+      <c r="L15" s="47">
+        <v>2.02</v>
+      </c>
+      <c r="M15" s="47">
+        <v>1.97</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C16" s="6">
-        <v>2</v>
+        <v>10.7</v>
       </c>
       <c r="D16" s="2">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="E16" s="2">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="F16" s="2">
         <f t="shared" si="0"/>
-        <v>2.2999999999999998</v>
+        <v>10.899999999999999</v>
       </c>
       <c r="G16" s="2">
         <f t="shared" si="1"/>
-        <v>1.7</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I16" s="47"/>
-      <c r="J16" s="47"/>
-      <c r="K16" s="47"/>
-      <c r="L16" s="47"/>
-      <c r="M16" s="47"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+        <v>10.5</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I16" s="47">
+        <v>10.58</v>
+      </c>
+      <c r="J16" s="47">
+        <v>10.65</v>
+      </c>
+      <c r="K16" s="47">
+        <v>10.62</v>
+      </c>
+      <c r="L16" s="47">
+        <v>10.72</v>
+      </c>
+      <c r="M16" s="47">
+        <v>10.61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C17" s="6">
-        <v>10.7</v>
+        <v>19.5</v>
       </c>
       <c r="D17" s="2">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E17" s="2">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="F17" s="2">
         <f t="shared" si="0"/>
-        <v>10.899999999999999</v>
+        <v>19.8</v>
       </c>
       <c r="G17" s="2">
         <f t="shared" si="1"/>
-        <v>10.5</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I17" s="47"/>
-      <c r="J17" s="47"/>
-      <c r="K17" s="47"/>
-      <c r="L17" s="47"/>
-      <c r="M17" s="47"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+        <v>19.2</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I17" s="47">
+        <v>19.43</v>
+      </c>
+      <c r="J17" s="47">
+        <v>19.489999999999998</v>
+      </c>
+      <c r="K17" s="47">
+        <v>19.510000000000002</v>
+      </c>
+      <c r="L17" s="47">
+        <v>19.510000000000002</v>
+      </c>
+      <c r="M17" s="47">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>19</v>
       </c>
       <c r="C18" s="6">
-        <v>19.5</v>
+        <v>5</v>
       </c>
       <c r="D18" s="2">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="E18" s="2">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="F18" s="2">
         <f t="shared" si="0"/>
-        <v>19.8</v>
+        <v>5.2</v>
       </c>
       <c r="G18" s="2">
         <f t="shared" si="1"/>
-        <v>19.2</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I18" s="47"/>
-      <c r="J18" s="47"/>
-      <c r="K18" s="47"/>
-      <c r="L18" s="47"/>
-      <c r="M18" s="47"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+        <v>4.8</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I18" s="47">
+        <v>4.8099999999999996</v>
+      </c>
+      <c r="J18" s="47">
+        <v>4.91</v>
+      </c>
+      <c r="K18" s="47">
+        <v>4.95</v>
+      </c>
+      <c r="L18" s="47">
+        <v>4.97</v>
+      </c>
+      <c r="M18" s="47">
+        <v>4.9000000000000004</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C19" s="6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D19" s="2">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E19" s="2">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="F19" s="2">
         <f t="shared" si="0"/>
-        <v>5.2</v>
+        <v>1.3</v>
       </c>
       <c r="G19" s="2">
         <f t="shared" si="1"/>
-        <v>4.8</v>
-      </c>
-      <c r="H19" s="3" t="s">
+        <v>0.7</v>
+      </c>
+      <c r="H19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I19" s="47"/>
-      <c r="J19" s="47"/>
-      <c r="K19" s="47"/>
-      <c r="L19" s="47"/>
-      <c r="M19" s="47"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="I19" s="47">
+        <v>3.1606000000000001</v>
+      </c>
+      <c r="J19" s="47">
+        <v>3.2361</v>
+      </c>
+      <c r="K19" s="47">
+        <v>3.1827000000000001</v>
+      </c>
+      <c r="L19" s="47">
+        <v>3.0240999999999998</v>
+      </c>
+      <c r="M19" s="47">
+        <v>3.0533000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C20" s="6">
-        <v>1</v>
+        <v>5.4</v>
       </c>
       <c r="D20" s="2">
-        <v>0.3</v>
+        <v>0.33700000000000002</v>
       </c>
       <c r="E20" s="2">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="F20" s="2">
         <f t="shared" si="0"/>
-        <v>1.3</v>
+        <v>5.7370000000000001</v>
       </c>
       <c r="G20" s="2">
         <f t="shared" si="1"/>
-        <v>0.7</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I20" s="47"/>
-      <c r="J20" s="47"/>
-      <c r="K20" s="47"/>
-      <c r="L20" s="47"/>
-      <c r="M20" s="47"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+        <v>5.4</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I20" s="47">
+        <v>5.5</v>
+      </c>
+      <c r="J20" s="47">
+        <v>5.49</v>
+      </c>
+      <c r="K20" s="47">
+        <v>5.52</v>
+      </c>
+      <c r="L20" s="47">
+        <v>5.53</v>
+      </c>
+      <c r="M20" s="47">
+        <v>5.51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C21" s="6">
-        <v>5.4</v>
+        <v>7.1</v>
       </c>
       <c r="D21" s="2">
-        <v>0.33700000000000002</v>
+        <v>0.2</v>
       </c>
       <c r="E21" s="2">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="F21" s="2">
         <f t="shared" si="0"/>
-        <v>5.7370000000000001</v>
+        <v>7.3</v>
       </c>
       <c r="G21" s="2">
         <f t="shared" si="1"/>
-        <v>5.4</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I21" s="47"/>
-      <c r="J21" s="47"/>
-      <c r="K21" s="47"/>
-      <c r="L21" s="47"/>
-      <c r="M21" s="47"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+        <v>6.8999999999999995</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I21" s="47">
+        <v>7.18</v>
+      </c>
+      <c r="J21" s="47">
+        <v>7.23</v>
+      </c>
+      <c r="K21" s="47">
+        <v>7.15</v>
+      </c>
+      <c r="L21" s="47">
+        <v>7.04</v>
+      </c>
+      <c r="M21" s="47">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C22" s="6">
-        <v>7.1</v>
+        <v>1.5</v>
       </c>
       <c r="D22" s="2">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E22" s="2">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="F22" s="2">
         <f t="shared" si="0"/>
-        <v>7.3</v>
+        <v>1.8</v>
       </c>
       <c r="G22" s="2">
         <f t="shared" si="1"/>
-        <v>6.8999999999999995</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>45</v>
+        <v>1.2</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="I22" s="47"/>
       <c r="J22" s="47"/>
@@ -2244,65 +2389,75 @@
       <c r="L22" s="47"/>
       <c r="M22" s="47"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C23" s="6">
-        <v>1.5</v>
+        <v>5.4</v>
       </c>
       <c r="D23" s="2">
-        <v>0.3</v>
+        <v>0.33700000000000002</v>
       </c>
       <c r="E23" s="2">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="F23" s="2">
         <f t="shared" si="0"/>
-        <v>1.8</v>
+        <v>5.7370000000000001</v>
       </c>
       <c r="G23" s="2">
         <f t="shared" si="1"/>
-        <v>1.2</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I23" s="47"/>
-      <c r="J23" s="47"/>
-      <c r="K23" s="47"/>
-      <c r="L23" s="47"/>
-      <c r="M23" s="47"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+        <v>5.4</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I23" s="47">
+        <v>5.49</v>
+      </c>
+      <c r="J23" s="47">
+        <v>5.53</v>
+      </c>
+      <c r="K23" s="47">
+        <v>5.55</v>
+      </c>
+      <c r="L23" s="47">
+        <v>5.54</v>
+      </c>
+      <c r="M23" s="47">
+        <v>5.53</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C24" s="6">
-        <v>5.4</v>
+        <v>1.5</v>
       </c>
       <c r="D24" s="2">
-        <v>0.33700000000000002</v>
+        <v>0.3</v>
       </c>
       <c r="E24" s="2">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="F24" s="2">
         <f t="shared" si="0"/>
-        <v>5.7370000000000001</v>
+        <v>1.8</v>
       </c>
       <c r="G24" s="2">
         <f t="shared" si="1"/>
-        <v>5.4</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>20</v>
+        <v>1.2</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="I24" s="47"/>
       <c r="J24" s="47"/>
@@ -2310,147 +2465,139 @@
       <c r="L24" s="47"/>
       <c r="M24" s="47"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C25" s="6">
-        <v>1.5</v>
+        <v>11</v>
       </c>
       <c r="D25" s="2">
-        <v>0.3</v>
-      </c>
-      <c r="E25" s="2">
-        <v>0.3</v>
+        <v>0</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="F25" s="2">
         <f t="shared" si="0"/>
-        <v>1.8</v>
+        <v>11</v>
       </c>
       <c r="G25" s="2">
-        <f t="shared" si="1"/>
-        <v>1.2</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I25" s="47"/>
-      <c r="J25" s="47"/>
-      <c r="K25" s="47"/>
-      <c r="L25" s="47"/>
-      <c r="M25" s="47"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I25" s="47">
+        <v>10.965999999999999</v>
+      </c>
+      <c r="J25" s="47">
+        <v>10.959</v>
+      </c>
+      <c r="K25" s="47">
+        <v>10.994</v>
+      </c>
+      <c r="L25" s="47">
+        <v>10.956</v>
+      </c>
+      <c r="M25" s="47">
+        <v>10.957000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C26" s="6">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D26" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E26" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="F26" s="2">
+        <f t="shared" ref="F26:F27" si="2">C26+D26</f>
+        <v>2.1</v>
+      </c>
+      <c r="G26" s="2">
+        <v>1</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I26" s="48">
+        <v>3.14</v>
+      </c>
+      <c r="J26" s="48">
+        <v>2.64</v>
+      </c>
+      <c r="K26" s="48">
+        <v>2.81</v>
+      </c>
+      <c r="L26" s="48">
+        <v>2.74</v>
+      </c>
+      <c r="M26" s="48">
+        <v>2.97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
+        <v>23</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="6">
+        <v>16</v>
+      </c>
+      <c r="D27" s="2">
         <v>0</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F26" s="2">
-        <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-      <c r="G26" s="2">
-        <v>0</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I26" s="47"/>
-      <c r="J26" s="47"/>
-      <c r="K26" s="47"/>
-      <c r="L26" s="47"/>
-      <c r="M26" s="47"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A27" s="4">
-        <v>22</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C27" s="6">
-        <v>2</v>
-      </c>
-      <c r="D27" s="2">
-        <v>0.1</v>
-      </c>
       <c r="E27" s="2">
-        <v>0.1</v>
+        <v>16</v>
       </c>
       <c r="F27" s="2">
-        <f t="shared" ref="F27:F28" si="2">C27+D27</f>
-        <v>2.1</v>
-      </c>
-      <c r="G27" s="2">
-        <v>1</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I27" s="48"/>
-      <c r="J27" s="48"/>
-      <c r="K27" s="48"/>
-      <c r="L27" s="48"/>
-      <c r="M27" s="48"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" s="4">
-        <v>23</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C28" s="6">
-        <v>16</v>
-      </c>
-      <c r="D28" s="2">
-        <v>0</v>
-      </c>
-      <c r="E28" s="2">
-        <v>16</v>
-      </c>
-      <c r="F28" s="2">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="G28" s="2">
+      <c r="G27" s="2">
         <v>0</v>
       </c>
-      <c r="H28" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I28" s="49"/>
-      <c r="J28" s="49"/>
-      <c r="K28" s="49"/>
-      <c r="L28" s="49"/>
-      <c r="M28" s="49"/>
+      <c r="H27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I27" s="49"/>
+      <c r="J27" s="49"/>
+      <c r="K27" s="49"/>
+      <c r="L27" s="49"/>
+      <c r="M27" s="49"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="Q31" s="1" t="s">
+        <v>45</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="G1:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:M28">
-    <cfRule type="cellIs" dxfId="19" priority="22" operator="notBetween">
+  <conditionalFormatting sqref="I5:M27">
+    <cfRule type="cellIs" dxfId="0" priority="22" operator="notBetween">
       <formula>$G5</formula>
       <formula>$F5</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="84" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="73" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>

</xml_diff>